<commit_message>
updated Mormugoa vessel at berth
</commit_message>
<xml_diff>
--- a/mormugao/raw_at_berth.xlsx
+++ b/mormugao/raw_at_berth.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,49 +431,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="n">
+      <c r="A1" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="n">
+      <c r="C1" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" t="n">
+      <c r="D1" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" t="n">
+      <c r="E1" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" t="n">
+      <c r="F1" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" t="n">
+      <c r="G1" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="H1" t="n">
+      <c r="H1" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="I1" t="n">
+      <c r="I1" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="J1" t="n">
+      <c r="J1" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="K1" t="n">
+      <c r="K1" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="L1" t="n">
+      <c r="L1" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="M1" t="n">
+      <c r="M1" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="N1" t="n">
+      <c r="N1" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="O1" t="n">
+      <c r="O1" s="1" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1115,49 +1127,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="n">
+      <c r="A1" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="n">
+      <c r="C1" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" t="n">
+      <c r="D1" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" t="n">
+      <c r="E1" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" t="n">
+      <c r="F1" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" t="n">
+      <c r="G1" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="H1" t="n">
+      <c r="H1" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="I1" t="n">
+      <c r="I1" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="J1" t="n">
+      <c r="J1" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="K1" t="n">
+      <c r="K1" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="L1" t="n">
+      <c r="L1" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="M1" t="n">
+      <c r="M1" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="N1" t="n">
+      <c r="N1" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="O1" t="n">
+      <c r="O1" s="1" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1814,49 +1826,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="n">
+      <c r="A1" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B1" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="n">
+      <c r="C1" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" t="n">
+      <c r="D1" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" t="n">
+      <c r="E1" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" t="n">
+      <c r="F1" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" t="n">
+      <c r="G1" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="H1" t="n">
+      <c r="H1" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="I1" t="n">
+      <c r="I1" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="J1" t="n">
+      <c r="J1" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="K1" t="n">
+      <c r="K1" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="L1" t="n">
+      <c r="L1" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="M1" t="n">
+      <c r="M1" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="N1" t="n">
+      <c r="N1" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="O1" t="n">
+      <c r="O1" s="1" t="n">
         <v>14</v>
       </c>
     </row>

</xml_diff>